<commit_message>
GITBOOK-5: Aggiornamento file excel
</commit_message>
<xml_diff>
--- a/docs/0OMsoqOg9GiJ2xusVHM2/.gitbook/assets/IO - Template servizi - Accesso civico agli atti.xlsx
+++ b/docs/0OMsoqOg9GiJ2xusVHM2/.gitbook/assets/IO - Template servizi - Accesso civico agli atti.xlsx
@@ -167,7 +167,7 @@
     <t>Utilizza il testo indicato per il pulsante. Inserisci il link alla pagina web che rimanda al servizio.</t>
   </si>
   <si>
-    <t>Presenta richiesta</t>
+    <t>Invia richiesta</t>
   </si>
   <si>
     <t>Link a termini e condizioni d'uso</t>
@@ -998,7 +998,7 @@
       <rPr>
         <b/>
       </rPr>
-      <t>Allegato (Premium)</t>
+      <t>Allegato</t>
     </r>
     <r>
       <rPr/>

</xml_diff>